<commit_message>
fix: apply verified guild popup and training simulator updates
</commit_message>
<xml_diff>
--- a/reports/빅딜/빅딜_training_mgf_report.xlsx
+++ b/reports/빅딜/빅딜_training_mgf_report.xlsx
@@ -1770,7 +1770,7 @@
     <t>https://mgf.gg/contents/character.php?n=%EB%B0%8D%EC%B8%84%ED%95%91</t>
   </si>
   <si>
-    <t>16조 2006억 7084만</t>
+    <t>16조 4918억 4615만</t>
   </si>
   <si>
     <t>걀보</t>
@@ -1791,6 +1791,15 @@
     <t>3조 5196억 4046만</t>
   </si>
   <si>
+    <t>랏뚜</t>
+  </si>
+  <si>
+    <t>https://mgf.gg/contents/character.php?n=%EB%9E%8F%EB%9A%9C</t>
+  </si>
+  <si>
+    <t>3조 1258억 3830만</t>
+  </si>
+  <si>
     <t>왕오이</t>
   </si>
   <si>
@@ -1800,13 +1809,13 @@
     <t>3조 78억 6848만</t>
   </si>
   <si>
-    <t>랏뚜</t>
-  </si>
-  <si>
-    <t>https://mgf.gg/contents/character.php?n=%EB%9E%8F%EB%9A%9C</t>
-  </si>
-  <si>
-    <t>2조 9878억 9689만</t>
+    <t>그냐앙</t>
+  </si>
+  <si>
+    <t>https://mgf.gg/contents/character.php?n=%EA%B7%B8%EB%83%90%EC%95%99</t>
+  </si>
+  <si>
+    <t>2조 6959억 3259만</t>
   </si>
   <si>
     <t>이호은</t>
@@ -1836,15 +1845,6 @@
     <t>2조 5975억 5879만</t>
   </si>
   <si>
-    <t>그냐앙</t>
-  </si>
-  <si>
-    <t>https://mgf.gg/contents/character.php?n=%EA%B7%B8%EB%83%90%EC%95%99</t>
-  </si>
-  <si>
-    <t>2조 5586억 3591만</t>
-  </si>
-  <si>
     <t>하깁s</t>
   </si>
   <si>
@@ -1860,7 +1860,7 @@
     <t>https://mgf.gg/contents/character.php?n=%EC%95%BC%EC%A0%9C</t>
   </si>
   <si>
-    <t>2조 3811억 4994만</t>
+    <t>2조 4181억 16만</t>
   </si>
   <si>
     <t>은디탁</t>
@@ -1896,7 +1896,7 @@
     <t>https://mgf.gg/contents/character.php?n=%EB%84%A4%EB%AA%A8%EC%88%98%EB%B0%95</t>
   </si>
   <si>
-    <t>1조 9032억 8552만</t>
+    <t>1조 9175억 6016만</t>
   </si>
   <si>
     <t>부라</t>
@@ -1905,7 +1905,7 @@
     <t>https://mgf.gg/contents/character.php?n=%EB%B6%80%EB%9D%BC</t>
   </si>
   <si>
-    <t>1조 4029억 9332만</t>
+    <t>1조 4308억 7074만</t>
   </si>
   <si>
     <t>늙은마</t>
@@ -1914,7 +1914,7 @@
     <t>https://mgf.gg/contents/character.php?n=%EB%8A%99%EC%9D%80%EB%A7%88</t>
   </si>
   <si>
-    <t>1조 3664억 3029만</t>
+    <t>1조 3816억 6012만</t>
   </si>
   <si>
     <t>라이언킹</t>
@@ -1932,7 +1932,7 @@
     <t>https://mgf.gg/contents/character.php?n=jinajina</t>
   </si>
   <si>
-    <t>1조 596억 5673만</t>
+    <t>1조 798억 1637만</t>
   </si>
   <si>
     <t>덕장이다습할</t>
@@ -1950,7 +1950,7 @@
     <t>https://mgf.gg/contents/character.php?n=%EC%BC%A0%EC%84%9D</t>
   </si>
   <si>
-    <t>9895억 7608만</t>
+    <t>1조 18억 5366만</t>
   </si>
   <si>
     <t>뿌베</t>
@@ -1959,7 +1959,7 @@
     <t>https://mgf.gg/contents/character.php?n=%EB%BF%8C%EB%B2%A0</t>
   </si>
   <si>
-    <t>8781억 6967만</t>
+    <t>8847억 5595만</t>
   </si>
   <si>
     <t>챵술사</t>
@@ -8278,10 +8278,10 @@
         <v>93</v>
       </c>
       <c r="G6" s="2" t="s">
-        <v>87</v>
+        <v>105</v>
       </c>
       <c r="H6" s="2" t="s">
-        <v>135</v>
+        <v>156</v>
       </c>
       <c r="I6" s="2" t="s">
         <v>588</v>
@@ -8310,10 +8310,10 @@
         <v>93</v>
       </c>
       <c r="G7" s="2" t="s">
-        <v>105</v>
+        <v>87</v>
       </c>
       <c r="H7" s="2" t="s">
-        <v>156</v>
+        <v>135</v>
       </c>
       <c r="I7" s="2" t="s">
         <v>591</v>
@@ -8342,10 +8342,10 @@
         <v>93</v>
       </c>
       <c r="G8" s="2" t="s">
-        <v>87</v>
+        <v>125</v>
       </c>
       <c r="H8" s="2" t="s">
-        <v>156</v>
+        <v>135</v>
       </c>
       <c r="I8" s="2" t="s">
         <v>594</v>
@@ -8374,10 +8374,10 @@
         <v>93</v>
       </c>
       <c r="G9" s="2" t="s">
-        <v>421</v>
+        <v>87</v>
       </c>
       <c r="H9" s="2" t="s">
-        <v>161</v>
+        <v>156</v>
       </c>
       <c r="I9" s="2" t="s">
         <v>597</v>
@@ -8406,10 +8406,10 @@
         <v>93</v>
       </c>
       <c r="G10" s="2" t="s">
-        <v>125</v>
+        <v>421</v>
       </c>
       <c r="H10" s="2" t="s">
-        <v>156</v>
+        <v>161</v>
       </c>
       <c r="I10" s="2" t="s">
         <v>600</v>
@@ -8441,7 +8441,7 @@
         <v>125</v>
       </c>
       <c r="H11" s="2" t="s">
-        <v>135</v>
+        <v>156</v>
       </c>
       <c r="I11" s="2" t="s">
         <v>603</v>

</xml_diff>